<commit_message>
supplier media integration complete
</commit_message>
<xml_diff>
--- a/frontend/mobile/assets/bulk-import/TRU_Connect_Product_Import_Template.xlsx
+++ b/frontend/mobile/assets/bulk-import/TRU_Connect_Product_Import_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Units" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Categories" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Units" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,8 +71,14 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -89,6 +95,16 @@
       <patternFill patternType="solid">
         <fgColor rgb="00757575"/>
         <bgColor rgb="00757575"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E7D32"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00757575"/>
       </patternFill>
     </fill>
   </fills>
@@ -118,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -136,6 +152,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -499,9 +518,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -509,187 +528,417 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>quantity</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>sku</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>compare_at_price</t>
+        </is>
+      </c>
+      <c r="I1" s="12" t="inlineStr">
         <is>
           <t>image_1</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="J1" s="12" t="inlineStr">
         <is>
           <t>image_2</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="K1" s="12" t="inlineStr">
         <is>
           <t>image_3</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="L1" s="12" t="inlineStr">
         <is>
           <t>image_4</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="M1" s="12" t="inlineStr">
         <is>
           <t>image_5</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>Coca-Cola 500ml</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>Beverages</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>12.00</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="13" t="inlineStr">
         <is>
           <t>Each</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="13" t="inlineStr">
         <is>
           <t>47</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="13" t="inlineStr">
+        <is>
+          <t>SKU-000001</t>
+        </is>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>Ice-cold 500ml bottle.</t>
+        </is>
+      </c>
+      <c r="H2" s="13" t="inlineStr">
+        <is>
+          <t>15.00</t>
+        </is>
+      </c>
+      <c r="I2" s="13" t="inlineStr">
         <is>
           <t>coke500.jpg</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="J2" s="13" t="inlineStr">
         <is>
           <t>coke500_back.jpg</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr"/>
-      <c r="I2" s="3" t="inlineStr"/>
-      <c r="J2" s="3" t="inlineStr"/>
+      <c r="K2" s="13" t="n"/>
+      <c r="L2" s="13" t="n"/>
+      <c r="M2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Simba Chips 120g</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Snacks &amp; Confectionery</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>18.50</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>Each</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="13" t="n"/>
+      <c r="G3" s="13" t="n"/>
+      <c r="H3" s="13" t="n"/>
+      <c r="I3" s="13" t="inlineStr">
         <is>
           <t>simba120.jpg</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
+      <c r="J3" s="13" t="n"/>
+      <c r="K3" s="13" t="n"/>
+      <c r="L3" s="13" t="n"/>
+      <c r="M3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Albany Bread</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Bakery</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>19.99</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Each</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="13" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Delete the 3 rows above before uploading -- they're examples only. Green headers are required, grey are optional.</t>
-        </is>
-      </c>
+      <c r="F4" s="13" t="n"/>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>Sliced white bread, 1 loaf per unit.</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="n"/>
+      <c r="I4" s="13" t="n"/>
+      <c r="J4" s="13" t="n"/>
+      <c r="K4" s="13" t="n"/>
+      <c r="L4" s="13" t="n"/>
+      <c r="M4" s="13" t="n"/>
     </row>
   </sheetData>
-  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>How to fill in this template</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Required. The product's full name, e.g. "Coca-Cola 500ml".</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Required. Must exactly match one of the names on the Categories sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Required. Rands, e.g. 12.00 or 12,00 -- no currency symbol needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Required. What the price is for -- must exactly match one of the names on the Units sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Optional. How many you currently have. Leave blank to start at 0 (Out of stock until you add stock).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>sku</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Optional. Your own tracking label. Leave blank and TRU Connect generates one for you automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Optional. Plain text shown to businesses when they order, e.g. "3 loaves per case."</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>compare_at_price</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Optional. The "was" price for a sale, e.g. 25.00. Must be higher than price, or the row will show an error. Leave blank if you're not running a sale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>image_1</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Optional. The exact filename of the main photo inside your images ZIP, e.g. "coke500.jpg".</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>image_2</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Optional. A second photo filename.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>image_3</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Optional. A third photo filename.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>image_4</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Optional. A fourth photo filename.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>image_5</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Optional. A fifth photo filename.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Images</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>If you're including photos, put them all in one ZIP file (no folders needed) and upload it alongside this spreadsheet. Each image_1 to image_5 value must exactly match a filename inside that ZIP, including the file extension (.jpg, .jpeg, .png, or .webp). Products without any image columns filled in will publish without a photo -- that's fine, you can add photos later.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -832,7 +1081,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -945,172 +1194,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:B18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>How to fill in this template</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>Required. The product's full name, e.g. "Coca-Cola 500ml".</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Required. Must exactly match one of the names on the Categories sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Required. Rands, e.g. 12.00 or 12,00 -- no currency symbol needed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Required. What the price is for -- must exactly match one of the names on the Units sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>Optional. How many you currently have. Leave blank to start at 0 (Out of stock until you add stock).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>image_1</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>Optional. The exact filename of the main photo inside your images ZIP, e.g. "coke500.jpg".</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>image_2</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Optional. A second photo filename.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>image_3</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Optional. A third photo filename.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>image_4</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Optional. A fourth photo filename.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>image_5</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Optional. A fifth photo filename.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>Images</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>If you're including photos, put them all in one ZIP file (no folders needed) and upload it alongside this spreadsheet. Each image_1 to image_5 value must exactly match a filename inside that ZIP, including the file extension (.jpg, .jpeg, .png, or .webp). Products without any image columns filled in will publish without a photo -- that's fine, you can add photos later.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B18"/>
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
-  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Regenerate the bulk-import template and guide
Both are built from IMPORT_FIELDS by scripts/generate_import_template.py,
so they were stale the moment barcode/brand/pack_quantity/pack_unit
were added to the importer. 17 columns now.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/mobile/assets/bulk-import/TRU_Connect_Product_Import_Template.xlsx
+++ b/frontend/mobile/assets/bulk-import/TRU_Connect_Product_Import_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Categories" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Units" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Units" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>